<commit_message>
added By Weight field in packaging screen
</commit_message>
<xml_diff>
--- a/template/Packaging_Template.xlsx
+++ b/template/Packaging_Template.xlsx
@@ -27,12 +27,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Packaging Name</t>
   </si>
   <si>
     <t>Packaging Type</t>
+  </si>
+  <si>
+    <t>By Weight</t>
   </si>
 </sst>
 </file>
@@ -995,7 +998,9 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1"/>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -1004,9 +1009,12 @@
       <c r="I1" s="1"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576">
       <formula1>"Original,Repack"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576">
+      <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>